<commit_message>
Finalize requirements review and update Appendix B
</commit_message>
<xml_diff>
--- a/assets/planning/BusinessRequirements_1.0.1.xlsx
+++ b/assets/planning/BusinessRequirements_1.0.1.xlsx
@@ -4,19 +4,20 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="30" windowWidth="14295" windowHeight="7695"/>
+    <workbookView xWindow="360" yWindow="30" windowWidth="14295" windowHeight="7695" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="BusinessReq" sheetId="1" r:id="rId1"/>
     <sheet name="Draft_Entities" sheetId="3" r:id="rId2"/>
     <sheet name="Req-P1-06" sheetId="7" r:id="rId3"/>
+    <sheet name="ReqReview" sheetId="8" r:id="rId4"/>
   </sheets>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="213">
   <si>
     <t>ID</t>
   </si>
@@ -592,13 +593,76 @@
   </si>
   <si>
     <t>We need to walk through the ordering process without submitting an order and capture</t>
+  </si>
+  <si>
+    <t>Final status</t>
+  </si>
+  <si>
+    <t>Implementation evidence and notes</t>
+  </si>
+  <si>
+    <t>Complete</t>
+  </si>
+  <si>
+    <t>CUSTOMER stores registered-customer information. Guest contact details are retained on ORDERS.</t>
+  </si>
+  <si>
+    <t>ADDRESS records are linked to CUSTOMER. A customer may maintain multiple addresses.</t>
+  </si>
+  <si>
+    <t>Each ORDERS record references one STORE through store_id.</t>
+  </si>
+  <si>
+    <t>MENU_CATEGORY and PRODUCT maintain the menu structure.</t>
+  </si>
+  <si>
+    <t>PRODUCT_VARIATION records the size, crust type, and base price for each product variation.</t>
+  </si>
+  <si>
+    <t>CUSTOMIZATION_OPTION defines valid options. ORDER_ITEM_CUSTOMIZATION preserves each charged adjustment.</t>
+  </si>
+  <si>
+    <t>ORDERS, ORDER_ITEM, and ORDER_ITEM_CUSTOMIZATION record selected items and customizations.</t>
+  </si>
+  <si>
+    <t>ORDER_ITEM retains quantity and unit_price for the submitted order.</t>
+  </si>
+  <si>
+    <t>ORDERS stores fulfillment_type. delivery_address_id is optional for pickup orders.</t>
+  </si>
+  <si>
+    <t>PAYMENT records method, amount, date, and status without full card details.</t>
+  </si>
+  <si>
+    <t>ORDER_STATUS_EVENT records dated status changes for each order.</t>
+  </si>
+  <si>
+    <t>PROMOTION defines offers. ORDER_PROMOTION records the promotion and discount applied to an order.</t>
+  </si>
+  <si>
+    <t>LOYALTY_ACCOUNT and LOYALTY_TRANSACTION record membership and point activity.</t>
+  </si>
+  <si>
+    <t>Ten business queries report on sales, products, customizations, stores, promotions, customers, loyalty, subscriptions, and fulfillment.</t>
+  </si>
+  <si>
+    <t>ORDER_ITEM, ORDER_PROMOTION, and SUBSCRIPTION_BENEFIT_EVENT retain values applied when an order was placed.</t>
+  </si>
+  <si>
+    <t>SUBSCRIPTION_PLAN stores plan price, billing cycle, benefit amount, usage limit, and active status.</t>
+  </si>
+  <si>
+    <t>CUSTOMER_SUBSCRIPTION records enrollment, status, start date, renewal date, and cancellation date.</t>
+  </si>
+  <si>
+    <t>SUBSCRIPTION_BENEFIT_EVENT links a subscription benefit to the order where it was redeemed.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -613,6 +677,14 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -622,12 +694,27 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -638,13 +725,18 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1832,4 +1924,344 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId9"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="B2:F20"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="3" max="3" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="70.42578125" customWidth="1"/>
+    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="71.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:6">
+      <c r="B2" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" ht="30">
+      <c r="B3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" ht="30">
+      <c r="B4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6">
+      <c r="B5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" ht="30">
+      <c r="B6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" ht="30">
+      <c r="B7" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" ht="30">
+      <c r="B8" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" ht="30">
+      <c r="B9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" ht="30">
+      <c r="B10" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6">
+      <c r="B11" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" ht="30">
+      <c r="B12" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" ht="30">
+      <c r="B13" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" ht="30">
+      <c r="B14" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" ht="30">
+      <c r="B15" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" ht="30">
+      <c r="B16" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" ht="30">
+      <c r="B17" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" ht="30">
+      <c r="B18" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" ht="30">
+      <c r="B19" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" ht="30">
+      <c r="B20" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>212</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>